<commit_message>
Updated notes being wonky for some reason
</commit_message>
<xml_diff>
--- a/Helldivers/Super Credits Log.xlsx
+++ b/Helldivers/Super Credits Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\python_projects\Helldivers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BC4928B-53F1-467F-BFA2-4CAA17DE1513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27E08ACD-1A74-405C-9944-27A6494ECAC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{3980E34F-3276-48B4-AAA9-72DB210AB7A4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="72">
   <si>
     <t>Mission Time</t>
   </si>
@@ -761,9 +761,7 @@
       <c r="M2" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N2" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N2" s="1"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -981,9 +979,7 @@
       <c r="M7" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N7" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N7" s="1"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -1025,9 +1021,7 @@
       <c r="M8" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N8" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N8" s="1"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -1069,9 +1063,7 @@
       <c r="M9" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N9" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N9" s="1"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -1113,9 +1105,7 @@
       <c r="M10" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N10" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N10" s="1"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
@@ -1157,9 +1147,7 @@
       <c r="M11" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N11" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N11" s="1"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
@@ -1201,9 +1189,7 @@
       <c r="M12" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N12" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N12" s="1"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
@@ -1245,9 +1231,7 @@
       <c r="M13" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N13" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N13" s="1"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
@@ -1289,9 +1273,7 @@
       <c r="M14" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N14" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N14" s="1"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
@@ -1333,9 +1315,7 @@
       <c r="M15" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N15" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N15" s="1"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
@@ -1377,9 +1357,7 @@
       <c r="M16" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N16" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N16" s="1"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
@@ -1421,9 +1399,7 @@
       <c r="M17" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N17" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N17" s="1"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
@@ -1465,9 +1441,7 @@
       <c r="M18" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N18" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N18" s="1"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
@@ -1509,9 +1483,7 @@
       <c r="M19" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N19" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N19" s="1"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
@@ -1641,9 +1613,7 @@
       <c r="M22" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N22" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N22" s="1"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
@@ -1773,9 +1743,7 @@
       <c r="M25">
         <v>440</v>
       </c>
-      <c r="N25" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N25" s="1"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
@@ -1817,9 +1785,7 @@
       <c r="M26">
         <v>440</v>
       </c>
-      <c r="N26" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N26" s="1"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
@@ -1861,9 +1827,7 @@
       <c r="M27">
         <v>440</v>
       </c>
-      <c r="N27" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N27" s="1"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
@@ -1905,9 +1869,7 @@
       <c r="M28">
         <v>450</v>
       </c>
-      <c r="N28" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N28" s="1"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
@@ -1949,9 +1911,7 @@
       <c r="M29">
         <v>480</v>
       </c>
-      <c r="N29" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N29" s="1"/>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
@@ -1993,9 +1953,7 @@
       <c r="M30">
         <v>480</v>
       </c>
-      <c r="N30" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N30" s="1"/>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
@@ -2037,9 +1995,7 @@
       <c r="M31">
         <v>480</v>
       </c>
-      <c r="N31" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N31" s="1"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
@@ -2081,9 +2037,7 @@
       <c r="M32">
         <v>480</v>
       </c>
-      <c r="N32" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N32" s="1"/>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
@@ -2125,9 +2079,7 @@
       <c r="M33">
         <v>480</v>
       </c>
-      <c r="N33" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N33" s="1"/>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
@@ -2169,9 +2121,7 @@
       <c r="M34">
         <v>480</v>
       </c>
-      <c r="N34" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N34" s="1"/>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
@@ -2213,9 +2163,7 @@
       <c r="M35">
         <v>480</v>
       </c>
-      <c r="N35" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N35" s="1"/>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
@@ -2257,9 +2205,7 @@
       <c r="M36">
         <v>480</v>
       </c>
-      <c r="N36" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N36" s="1"/>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
@@ -2301,9 +2247,7 @@
       <c r="M37">
         <v>500</v>
       </c>
-      <c r="N37" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N37" s="1"/>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
@@ -2345,9 +2289,7 @@
       <c r="M38">
         <v>510</v>
       </c>
-      <c r="N38" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N38" s="1"/>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
@@ -2433,9 +2375,7 @@
       <c r="M40">
         <v>520</v>
       </c>
-      <c r="N40" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N40" s="1"/>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
@@ -2565,9 +2505,7 @@
       <c r="M43">
         <v>540</v>
       </c>
-      <c r="N43" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N43" s="1"/>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
@@ -2609,9 +2547,7 @@
       <c r="M44">
         <v>540</v>
       </c>
-      <c r="N44" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N44" s="1"/>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
@@ -2697,9 +2633,7 @@
       <c r="M46">
         <v>570</v>
       </c>
-      <c r="N46" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N46" s="1"/>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="4">
@@ -2829,9 +2763,7 @@
       <c r="M49">
         <v>570</v>
       </c>
-      <c r="N49" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N49" s="1"/>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="4">
@@ -2917,9 +2849,7 @@
       <c r="M51">
         <v>570</v>
       </c>
-      <c r="N51" s="1" t="s">
-        <v>36</v>
-      </c>
+      <c r="N51" s="1"/>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="4">
@@ -3049,9 +2979,7 @@
       <c r="M54">
         <v>570</v>
       </c>
-      <c r="N54" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N54" s="1"/>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="4">
@@ -3093,9 +3021,7 @@
       <c r="M55">
         <v>580</v>
       </c>
-      <c r="N55" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N55" s="1"/>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="4">
@@ -3137,9 +3063,7 @@
       <c r="M56">
         <v>620</v>
       </c>
-      <c r="N56" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N56" s="1"/>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="4">
@@ -3225,9 +3149,7 @@
       <c r="M58">
         <v>630</v>
       </c>
-      <c r="N58" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N58" s="1"/>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" s="4">
@@ -3445,9 +3367,7 @@
       <c r="M63">
         <v>240</v>
       </c>
-      <c r="N63" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N63" s="1"/>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="4">
@@ -3489,9 +3409,7 @@
       <c r="M64">
         <v>240</v>
       </c>
-      <c r="N64" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N64" s="1"/>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="4">
@@ -3533,9 +3451,7 @@
       <c r="M65">
         <v>240</v>
       </c>
-      <c r="N65" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N65" s="1"/>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="4">
@@ -3577,9 +3493,7 @@
       <c r="M66">
         <v>240</v>
       </c>
-      <c r="N66" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N66" s="1"/>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67" s="4">
@@ -3621,9 +3535,7 @@
       <c r="M67">
         <v>240</v>
       </c>
-      <c r="N67" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N67" s="1"/>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="4">
@@ -3665,9 +3577,7 @@
       <c r="M68">
         <v>240</v>
       </c>
-      <c r="N68" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N68" s="1"/>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69" s="4">
@@ -3709,9 +3619,7 @@
       <c r="M69">
         <v>240</v>
       </c>
-      <c r="N69" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N69" s="1"/>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" s="4">
@@ -3753,9 +3661,7 @@
       <c r="M70">
         <v>240</v>
       </c>
-      <c r="N70" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N70" s="1"/>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" s="4">
@@ -3797,9 +3703,7 @@
       <c r="M71">
         <v>240</v>
       </c>
-      <c r="N71" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N71" s="1"/>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" s="4">
@@ -3841,9 +3745,7 @@
       <c r="M72">
         <v>240</v>
       </c>
-      <c r="N72" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N72" s="1"/>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" s="4">
@@ -3929,9 +3831,7 @@
       <c r="M74">
         <v>260</v>
       </c>
-      <c r="N74" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="N74" s="1"/>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A75" s="4">

</xml_diff>